<commit_message>
Added challenge 4 explanation (number 82)
</commit_message>
<xml_diff>
--- a/Solution explanations.xlsx
+++ b/Solution explanations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ainis\Desktop\LIFE\Coding projects\Daily challanges\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20F8C495-5F3B-4F2B-9D45-EE7A0FE3E043}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCCC5494-B048-4EFD-BB01-1DC6C0384A56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BDCE91D3-EC99-46FF-ABB3-2304E474D35E}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="167">
   <si>
     <t>Problem name</t>
   </si>
@@ -534,6 +534,12 @@
   </si>
   <si>
     <t>We set the goal to the end index, be begin iterating from the index before the goal and check if we can move the goal index closer to 0, lastly we check if its eqaul to 0</t>
+  </si>
+  <si>
+    <t>Jump Game II</t>
+  </si>
+  <si>
+    <t>We  set the current index to 0, we get the current jump size and find the index that gives the furthest jump possible (j + nums[j]) and we move to that one</t>
   </si>
 </sst>
 </file>
@@ -2743,10 +2749,14 @@
       <c r="B86" s="1">
         <v>82</v>
       </c>
-      <c r="C86" s="2"/>
-      <c r="D86" s="2"/>
-      <c r="E86" s="2"/>
-      <c r="F86" s="3"/>
+      <c r="C86" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="D86" s="5"/>
+      <c r="E86" s="5"/>
+      <c r="F86" s="3" t="s">
+        <v>166</v>
+      </c>
       <c r="G86" s="3"/>
       <c r="H86" s="3"/>
       <c r="I86" s="3"/>

</xml_diff>

<commit_message>
Added challenge 15 explanation (number 122)
</commit_message>
<xml_diff>
--- a/Solution explanations.xlsx
+++ b/Solution explanations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ainis\Desktop\LIFE\Coding projects\Daily challanges\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE86198F-9CAE-4DB9-B1B4-A3580A261561}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B96E72A3-094F-4969-9631-2AE1ED019ACC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BDCE91D3-EC99-46FF-ABB3-2304E474D35E}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="247">
   <si>
     <t>Problem name</t>
   </si>
@@ -774,6 +774,12 @@
   </si>
   <si>
     <t>We use a BFS algorithm, where we explore each level, but only add the last node's value (left to right) to the result array</t>
+  </si>
+  <si>
+    <t>Construct Quad Tree</t>
+  </si>
+  <si>
+    <t>We create a recursive algorithm, that checks if all n by n squares are the same, if so we return a node that is marked as a leaf, if not all nodes match, we divide the grid into four subGrids searching for sections that can resemble a leaf node, we continue recursively until the entire grid has been searched</t>
   </si>
 </sst>
 </file>
@@ -864,7 +870,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -888,9 +894,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -3796,7 +3799,7 @@
       <c r="B125" s="1">
         <v>121</v>
       </c>
-      <c r="C125" s="9" t="s">
+      <c r="C125" s="3" t="s">
         <v>243</v>
       </c>
       <c r="D125" s="3"/>
@@ -3817,10 +3820,14 @@
       <c r="B126" s="1">
         <v>122</v>
       </c>
-      <c r="C126" s="8"/>
-      <c r="D126" s="8"/>
-      <c r="E126" s="8"/>
-      <c r="F126" s="2"/>
+      <c r="C126" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="D126" s="3"/>
+      <c r="E126" s="3"/>
+      <c r="F126" s="2" t="s">
+        <v>246</v>
+      </c>
       <c r="G126" s="2"/>
       <c r="H126" s="2"/>
       <c r="I126" s="2"/>

</xml_diff>